<commit_message>
eloqwnt roadmap: rebuild deck + workbook with cleaned article titles
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/eloqwnt/keyword-research.xlsx
+++ b/decks/eloqwnt/keyword-research.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Branding Services: Scope, Timeline &amp; Cost</t>
+          <t>Branding Services: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B2B Content Marketing: What Actually Works</t>
+          <t>B2B Content Marketing: A Modern Take for B2B</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Getting SEO Web Design Right</t>
+          <t>Rethinking SEO Web Design for SaaS</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Leading Branding Agencies: Red Flags to Watch For</t>
+          <t>Leading Branding Agencies: A Vetting Checklist</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>UX Consulting Services: Questions to Ask First</t>
+          <t>UX Consulting Services: A B2B Buyer's Guide</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Branding and Marketing Strategy for Scaling Tech Brands</t>
+          <t>Rethinking Branding and Marketing Strategy for SaaS</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Digital Product Design Services: Scope, Timeline &amp; Cost</t>
+          <t>Digital Product Design Services: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Web App Design Services: Red Flags to Watch For</t>
+          <t>Web App Design Services: A Vetting Checklist</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Search Engine Optimization Landing Page: A B2B Guide for 2026</t>
+          <t>SEO Landing Pages: A B2B Guide for 2026</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Getting Website Planning Right</t>
+          <t>Website Planning: A B2B Guide for 2026</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SaaS Website for Scaling Tech Brands</t>
+          <t>SaaS Website, Explained for SaaS Teams</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Landing Page Design Best Practices: What Separates the Best</t>
+          <t>Landing Page Design Best Practices: Examples Worth Stealing</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Retail Branding: Lessons From High-Growth SaaS</t>
+          <t>Retail Branding: The Fundamentals</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Healthcare UX Design: What Actually Works</t>
+          <t>Healthcare UX Design, Explained for SaaS Teams</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Web Design Agency Pricing: What to Expect &amp; Pricing</t>
+          <t>Web Design Agency Pricing: Scope, Timeline &amp; Cost</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Benchmarking Form Wizard UX for B2B Tech</t>
+          <t>Form Wizard UX: What Separates the Best</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Comparing Top UX Firms for SaaS Teams</t>
+          <t>Top UX Firms: What Good Looks Like</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Family Branding Examples: Examples Worth Stealing</t>
+          <t>Family Branding Examples: A Side-by-Side Look</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SEO Web Design Packages: What Actually Works</t>
+          <t>SEO Web Design Packages: The Fundamentals</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SaaS Conversion Rates: Lessons From High-Growth SaaS</t>
+          <t>Getting SaaS Conversion Rates Right</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>A Founder's Guide to Brand Logotype</t>
+          <t>The Practical Guide to Brand Logotype</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Healthcare Branding: Lessons From High-Growth SaaS</t>
+          <t>Healthcare Branding: What Actually Works</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Brand Extension, Explained for SaaS Teams</t>
+          <t>Brand Extension for Scaling Tech Brands</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>The Practical Guide to Corporate Branding</t>
+          <t>A Founder's Guide to Corporate Branding</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Working With Top Branding Agencies: What to Know</t>
+          <t>Top Branding Agencies: What Working Together Looks Like</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Brand Consultancy: A Side-by-Side Look</t>
+          <t>Brand Consultancy: Examples Worth Stealing</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>B2B Brand Strategy: What Actually Works</t>
+          <t>B2B Brand Strategy: Lessons From High-Growth SaaS</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Getting Startup Branding Right</t>
+          <t>Startup Branding: A Modern Take for B2B</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>The Practical Guide to Website Packages</t>
+          <t>Rethinking Website Packages for SaaS</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Web Design and SEO Marketing: What Actually Works</t>
+          <t>Getting Web Design and SEO Marketing Right</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Vertical Slider UI, Explained for SaaS Teams</t>
+          <t>Vertical Slider UI: A B2B Guide for 2026</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Getting Landing Page Conversion Rate Right</t>
+          <t>Landing Page Conversion Rate for Scaling Tech Brands</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Mobile UX Design Agency: Questions to Ask First</t>
+          <t>Mobile UX Design Agency: Scope, Timeline &amp; Cost</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Slide Button UI: Lessons From High-Growth SaaS</t>
+          <t>Slide Button UI for Scaling Tech Brands</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Best UX Design Firms: What Separates the Best</t>
+          <t>Benchmarking Best UX Design Firms for B2B Tech</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CX vs UX: What Good Looks Like</t>
+          <t>CX vs UX, Ranked for Founders</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -3880,7 +3880,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Landing Page Copywriting for Scaling Tech Brands</t>
+          <t>Landing Page Copywriting: Lessons From High-Growth SaaS</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tooltip Alternatives UI Design Patterns: The Standouts Worth Studying</t>
+          <t>Comparing Tooltip Alternatives UI Design Patterns for SaaS Teams</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4012,7 +4012,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Getting Website Conversion Strategy Right</t>
+          <t>Website Conversion Strategy, Explained for SaaS Teams</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>B2B Growth Marketing Strategy for Scaling Tech Brands</t>
+          <t>B2B Growth Marketing Strategy: What Actually Works</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Working With B2B Content Marketing Consultant: What to Know</t>
+          <t>B2B Content Marketing Consultant: Questions to Ask First</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4144,7 +4144,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Working With UX Design Agency: What to Know</t>
+          <t>UX Design Agency: A Vetting Checklist</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Branding Kit: A B2B Guide for 2026</t>
+          <t>Getting Branding Kit Right</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4320,7 +4320,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>UX Design Company: Red Flags to Watch For</t>
+          <t>UX Design Company: What Working Together Looks Like</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>UI UX Agency: What to Expect &amp; Pricing</t>
+          <t>UI UX Agency: Red Flags to Watch For</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4452,7 +4452,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SEO Friendly Web Design for Scaling Tech Brands</t>
+          <t>SEO Friendly Web Design: The Fundamentals</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>UI/UX Design Agency: How to Brief the Right Partner</t>
+          <t>UI/UX Design Agency: Scope, Timeline &amp; Cost</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Brand Kit Examples: Examples Worth Stealing</t>
+          <t>Brand Kit Examples: A Side-by-Side Look</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Corporate Branding Services: What to Expect &amp; Pricing</t>
+          <t>Corporate Branding Services: What Working Together Looks Like</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -4716,7 +4716,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Website Development SEO: Lessons From High-Growth SaaS</t>
+          <t>Website Development SEO, Explained for SaaS Teams</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>User Interface Design Agency: What to Expect &amp; Pricing</t>
+          <t>User Interface Design Agency: What Working Together Looks Like</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>UI and UX Design Services: How to Brief the Right Partner</t>
+          <t>UI and UX Design Services: What to Expect &amp; Pricing</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>SEO Website Designer, Explained for SaaS Teams</t>
+          <t>SEO Website Designer: What Actually Works</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Mobile App Design Agency: A Vetting Checklist</t>
+          <t>Mobile App Design Agency: How to Brief the Right Partner</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -4980,7 +4980,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Getting User Experience Optimization Right</t>
+          <t>User Experience Optimization: What Actually Works</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Website Development Process: What Actually Works</t>
+          <t>Website Development Process: The Fundamentals</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Branding Agency Startups: A Vetting Checklist</t>
+          <t>Branding Agencies for Startups: A Vetting Checklist</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>UI/UX Design Services Company: Scope, Timeline &amp; Cost</t>
+          <t>UI/UX Design Services Company: Red Flags to Watch For</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Card UI, Explained for SaaS Teams</t>
+          <t>Card UI: Lessons From High-Growth SaaS</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>UI Design Examples: A Side-by-Side Look</t>
+          <t>The UI Design Examples Shortlist for B2B Founders</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Working With B2B UX Design Agency: What to Know</t>
+          <t>B2B UX Design Agency: Questions to Ask First</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>The Filter UI Shortlist for B2B Founders</t>
+          <t>Filter UI: Examples Worth Stealing</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -5464,7 +5464,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Event Landing Page, Explained for SaaS Teams</t>
+          <t>Event Landing Page: A Modern Take for B2B</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Webflow Development Services: How to Brief the Right Partner</t>
+          <t>Webflow Development Services: Red Flags to Watch For</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -5552,7 +5552,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Calendar UI for Scaling Tech Brands</t>
+          <t>Getting Calendar UI Right</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Examples of UI Pagination, Ranked for Founders</t>
+          <t>UI Pagination Patterns: Examples Worth Studying</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Best B2B Content Marketing Agency: A Vetting Checklist</t>
+          <t>Best B2B Content Marketing Agency: How to Brief the Right Partner</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Landing Page SEO Optimization: Lessons From High-Growth SaaS</t>
+          <t>Landing Page SEO Optimization: A Modern Take for B2B</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Landing Page Conversion Optimization, Explained for SaaS Teams</t>
+          <t>Rethinking Landing Page Conversion Optimization for SaaS</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Popover Examples UX: Examples Worth Stealing</t>
+          <t>Popover Examples UX: The Standouts Worth Studying</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">

</xml_diff>